<commit_message>
Build Q2406 PostgreSQL Client Windows task
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R3c5d20c6f4284b66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R81b50a472e82425b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -314,7 +314,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>边缘发布组导出的虚构通道、窗口、排队请求、事务计划、窗口合同和SQL骨架</x:v>
+        <x:v>边缘发布组从本轮排程导出的通道、窗口、排队请求、事务计划和窗口合同，以及数据库团队提供的SQL骨架</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>